<commit_message>
Archive STM32-aligned joystick, car upload tool, and notes.
Keep a rollback point for the handle mapping, deploy script, and competition docs. Local car credentials stay gitignored.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/1 WonderEchoPro/附录/命令词播报词协议列表V3_中文_RAICOM比赛.xlsx
+++ b/1 WonderEchoPro/附录/命令词播报词协议列表V3_中文_RAICOM比赛.xlsx
@@ -1425,39 +1425,13 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="26" t="n">
-        <v>3</v>
-      </c>
-      <c r="B5" s="27" t="inlineStr">
-        <is>
-          <t>你好小虎</t>
-        </is>
-      </c>
-      <c r="C5" s="26" t="inlineStr">
-        <is>
-          <t>唤醒词</t>
-        </is>
-      </c>
-      <c r="D5" s="27" t="inlineStr">
-        <is>
-          <t>我在</t>
-        </is>
-      </c>
-      <c r="E5" s="26" t="inlineStr">
-        <is>
-          <t>主</t>
-        </is>
-      </c>
-      <c r="F5" s="27" t="inlineStr">
-        <is>
-          <t>AA 55 03 00 FB</t>
-        </is>
-      </c>
-      <c r="G5" s="27" t="inlineStr">
-        <is>
-          <t>AA 55 03 00 FB</t>
-        </is>
-      </c>
+      <c r="A5" s="26" t="n"/>
+      <c r="B5" s="27" t="n"/>
+      <c r="C5" s="26" t="n"/>
+      <c r="D5" s="27" t="n"/>
+      <c r="E5" s="26" t="n"/>
+      <c r="F5" s="27" t="n"/>
+      <c r="G5" s="27" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="24" t="n">

</xml_diff>